<commit_message>
Auto-opdater EPGOAL 2026-10-07 15:17:21
</commit_message>
<xml_diff>
--- a/reports/tv3_tv3plus_fix_report.xlsx
+++ b/reports/tv3_tv3plus_fix_report.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TV3-TV3plus Fix'!$A$1:$E$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TV3-TV3plus Fix'!$A$1:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -489,7 +489,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>FORSLAG</t>
+          <t>SKRIVES</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>FORSLAG</t>
+          <t>SKRIVES</t>
         </is>
       </c>
     </row>
@@ -543,7 +543,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>FORSLAG</t>
+          <t>SKRIVES</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>FORSLAG</t>
+          <t>SKRIVES</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>FORSLAG</t>
+          <t>SKRIVES</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>FORSLAG</t>
+          <t>SKRIVES</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>FORSLAG</t>
+          <t>SKRIVES</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>FORSLAG</t>
+          <t>SKRIVES</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>FORSLAG</t>
+          <t>SKRIVES</t>
         </is>
       </c>
     </row>
@@ -732,39 +732,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>FORSLAG</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Sammenlagte kanal-ID'er (gammel reference)</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>TV3+ Denmark (DK, DA).dk, TV3+ HD (D) (T).dk, TV3+.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>FORSLAG</t>
+          <t>SKRIVES</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E12"/>
+  <autoFilter ref="A1:E11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -786,7 +759,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-06 15:56:27</t>
+          <t>2026-10-07 15:14:01</t>
         </is>
       </c>
     </row>
@@ -810,7 +783,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DRY-RUN</t>
+          <t>APPLY</t>
         </is>
       </c>
     </row>
@@ -821,7 +794,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>